<commit_message>
Clean up design doc and unassigned abilities
</commit_message>
<xml_diff>
--- a/docs/design/pokemon_romhack_tracker.xlsx
+++ b/docs/design/pokemon_romhack_tracker.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10322" uniqueCount="3566">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10332" uniqueCount="3576">
   <si>
     <t>Dex #</t>
   </si>
@@ -10740,6 +10740,36 @@
   </si>
   <si>
     <t>This Pokémon’s Sp. Atk is doubled. Its moves always gain same-type attack bonus.</t>
+  </si>
+  <si>
+    <t>The first Grass move after switch-in also uses Smack Down.</t>
+  </si>
+  <si>
+    <t>Poison moves hit twice. The second hit deals 40% damage.</t>
+  </si>
+  <si>
+    <t>Pulse moves lower the target's Sp. Def by 1.</t>
+  </si>
+  <si>
+    <t>If hit for 25% HP or less by a move, set Stealth Rock.</t>
+  </si>
+  <si>
+    <t>Sound moves used by this Pokemon also use Charge.</t>
+  </si>
+  <si>
+    <t>Below half HP, Flying moves restore 1/4 of the damage dealt.</t>
+  </si>
+  <si>
+    <t>If all party Pokemon share a type, set Misty Terrain.</t>
+  </si>
+  <si>
+    <t>If all party Pokemon share a type, set Psychic Terrain.</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Regular Mega ability is Delta Stream; no unique ability is currently mapped.</t>
   </si>
 </sst>
 </file>
@@ -76679,9 +76709,9 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:V191"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" ns3:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="14.6640625" customWidth="1"/>
@@ -76720,7 +76750,7 @@
     <col min="48" max="51" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:22" ht="28" customHeight="1" ns3:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -76788,7 +76818,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:22" ns3:dyDescent="0.2">
       <c r="A2" s="8">
         <v>3</v>
       </c>
@@ -76835,17 +76865,19 @@
         <v>6</v>
       </c>
       <c r="Q2" s="70" t="s">
-        <v>27</v>
+        <v>3002</v>
       </c>
       <c r="R2" t="s">
-        <v>28</v>
-      </c>
-      <c r="S2" s="11"/>
+        <v>3566</v>
+      </c>
+      <c r="S2" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T2" s="10"/>
       <c r="U2" s="11"/>
       <c r="V2" s="11"/>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:22" ns3:dyDescent="0.2">
       <c r="A3" s="8">
         <v>6</v>
       </c>
@@ -76897,12 +76929,14 @@
       <c r="R3" t="s">
         <v>37</v>
       </c>
-      <c r="S3" s="11"/>
+      <c r="S3" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T3" s="10"/>
       <c r="U3" s="11"/>
       <c r="V3" s="11"/>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:22" ns3:dyDescent="0.2">
       <c r="A4" s="8">
         <v>6</v>
       </c>
@@ -76954,12 +76988,14 @@
       <c r="R4" t="s">
         <v>37</v>
       </c>
-      <c r="S4" s="11"/>
+      <c r="S4" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T4" s="10"/>
       <c r="U4" s="11"/>
       <c r="V4" s="11"/>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:22" ns3:dyDescent="0.2">
       <c r="A5" s="8">
         <v>9</v>
       </c>
@@ -77009,12 +77045,14 @@
       <c r="R5" t="s">
         <v>46</v>
       </c>
-      <c r="S5" s="11"/>
+      <c r="S5" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T5" s="10"/>
       <c r="U5" s="11"/>
       <c r="V5" s="11"/>
     </row>
-    <row r="6" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:22" ht="16" ns3:dyDescent="0.2">
       <c r="A6" s="8">
         <v>15</v>
       </c>
@@ -77061,17 +77099,19 @@
         <v>6</v>
       </c>
       <c r="Q6" s="70" t="s">
-        <v>61</v>
+        <v>3081</v>
       </c>
       <c r="R6" s="71" t="s">
-        <v>62</v>
-      </c>
-      <c r="S6" s="11"/>
+        <v>3567</v>
+      </c>
+      <c r="S6" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T6" s="10"/>
       <c r="U6" s="11"/>
       <c r="V6" s="11"/>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:22" ns3:dyDescent="0.2">
       <c r="A7" s="8">
         <v>18</v>
       </c>
@@ -77123,12 +77163,14 @@
       <c r="R7" t="s">
         <v>73</v>
       </c>
-      <c r="S7" s="11"/>
+      <c r="S7" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T7" s="10"/>
       <c r="U7" s="11"/>
       <c r="V7" s="11"/>
     </row>
-    <row r="8" spans="1:22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:22" ht="16" customHeight="1" ns3:dyDescent="0.2">
       <c r="A8" s="8">
         <v>19</v>
       </c>
@@ -77189,7 +77231,7 @@
       <c r="U8" s="11"/>
       <c r="V8" s="11"/>
     </row>
-    <row r="9" spans="1:22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:22" ht="16" customHeight="1" ns3:dyDescent="0.2">
       <c r="A9" s="8">
         <v>20</v>
       </c>
@@ -77250,7 +77292,7 @@
       <c r="U9" s="11"/>
       <c r="V9" s="11"/>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:22" ns3:dyDescent="0.2">
       <c r="A10" s="8">
         <v>25</v>
       </c>
@@ -77307,7 +77349,7 @@
       <c r="U10" s="11"/>
       <c r="V10" s="11"/>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:22" ns3:dyDescent="0.2">
       <c r="A11" s="8">
         <v>26</v>
       </c>
@@ -77364,7 +77406,7 @@
       <c r="U11" s="11"/>
       <c r="V11" s="11"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:22" ns3:dyDescent="0.2">
       <c r="A12" s="8">
         <v>27</v>
       </c>
@@ -77423,7 +77465,7 @@
       <c r="U12" s="11"/>
       <c r="V12" s="11"/>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:22" ns3:dyDescent="0.2">
       <c r="A13" s="8">
         <v>28</v>
       </c>
@@ -77482,7 +77524,7 @@
       <c r="U13" s="11"/>
       <c r="V13" s="11"/>
     </row>
-    <row r="14" spans="1:22" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:22" ht="18" customHeight="1" ns3:dyDescent="0.2">
       <c r="A14" s="8">
         <v>37</v>
       </c>
@@ -77539,7 +77581,7 @@
       <c r="U14" s="11"/>
       <c r="V14" s="11"/>
     </row>
-    <row r="15" spans="1:22" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:22" ht="19" customHeight="1" ns3:dyDescent="0.2">
       <c r="A15" s="8">
         <v>38</v>
       </c>
@@ -77598,7 +77640,7 @@
       <c r="U15" s="11"/>
       <c r="V15" s="11"/>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:22" ns3:dyDescent="0.2">
       <c r="A16" s="8">
         <v>50</v>
       </c>
@@ -77659,7 +77701,7 @@
       <c r="U16" s="11"/>
       <c r="V16" s="11"/>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:22" ns3:dyDescent="0.2">
       <c r="A17" s="8">
         <v>51</v>
       </c>
@@ -77720,7 +77762,7 @@
       <c r="U17" s="11"/>
       <c r="V17" s="11"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:22" ns3:dyDescent="0.2">
       <c r="A18" s="8">
         <v>52</v>
       </c>
@@ -77779,7 +77821,7 @@
       <c r="U18" s="11"/>
       <c r="V18" s="11"/>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:22" ns3:dyDescent="0.2">
       <c r="A19" s="8">
         <v>52</v>
       </c>
@@ -77838,7 +77880,7 @@
       <c r="U19" s="11"/>
       <c r="V19" s="11"/>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:22" ns3:dyDescent="0.2">
       <c r="A20" s="8">
         <v>53</v>
       </c>
@@ -77897,7 +77939,7 @@
       <c r="U20" s="11"/>
       <c r="V20" s="11"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:22" ns3:dyDescent="0.2">
       <c r="A21" s="8">
         <v>58</v>
       </c>
@@ -77958,7 +78000,7 @@
       <c r="U21" s="11"/>
       <c r="V21" s="11"/>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:22" ns3:dyDescent="0.2">
       <c r="A22" s="8">
         <v>59</v>
       </c>
@@ -78019,7 +78061,7 @@
       <c r="U22" s="11"/>
       <c r="V22" s="11"/>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:22" ns3:dyDescent="0.2">
       <c r="A23" s="8">
         <v>65</v>
       </c>
@@ -78069,12 +78111,14 @@
       <c r="R23" t="s">
         <v>202</v>
       </c>
-      <c r="S23" s="11"/>
+      <c r="S23" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T23" s="10"/>
       <c r="U23" s="11"/>
       <c r="V23" s="11"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:22" ns3:dyDescent="0.2">
       <c r="A24" s="8">
         <v>74</v>
       </c>
@@ -78135,7 +78179,7 @@
       <c r="U24" s="11"/>
       <c r="V24" s="11"/>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:22" ns3:dyDescent="0.2">
       <c r="A25" s="8">
         <v>75</v>
       </c>
@@ -78196,7 +78240,7 @@
       <c r="U25" s="11"/>
       <c r="V25" s="11"/>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:22" ns3:dyDescent="0.2">
       <c r="A26" s="8">
         <v>76</v>
       </c>
@@ -78257,7 +78301,7 @@
       <c r="U26" s="11"/>
       <c r="V26" s="11"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:22" ns3:dyDescent="0.2">
       <c r="A27" s="8">
         <v>77</v>
       </c>
@@ -78316,7 +78360,7 @@
       <c r="U27" s="11"/>
       <c r="V27" s="11"/>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:22" ns3:dyDescent="0.2">
       <c r="A28" s="8">
         <v>78</v>
       </c>
@@ -78377,7 +78421,7 @@
       <c r="U28" s="11"/>
       <c r="V28" s="11"/>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:22" ns3:dyDescent="0.2">
       <c r="A29" s="8">
         <v>79</v>
       </c>
@@ -78436,7 +78480,7 @@
       <c r="U29" s="11"/>
       <c r="V29" s="11"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:22" ns3:dyDescent="0.2">
       <c r="A30" s="8">
         <v>80</v>
       </c>
@@ -78497,7 +78541,7 @@
       <c r="U30" s="11"/>
       <c r="V30" s="11"/>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:22" ns3:dyDescent="0.2">
       <c r="A31" s="8">
         <v>80</v>
       </c>
@@ -78549,12 +78593,14 @@
       <c r="R31" t="s">
         <v>240</v>
       </c>
-      <c r="S31" s="11"/>
+      <c r="S31" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T31" s="10"/>
       <c r="U31" s="11"/>
       <c r="V31" s="11"/>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:22" ns3:dyDescent="0.2">
       <c r="A32" s="8">
         <v>83</v>
       </c>
@@ -78611,7 +78657,7 @@
       <c r="U32" s="11"/>
       <c r="V32" s="11"/>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:22" ns3:dyDescent="0.2">
       <c r="A33" s="8">
         <v>88</v>
       </c>
@@ -78672,7 +78718,7 @@
       <c r="U33" s="11"/>
       <c r="V33" s="11"/>
     </row>
-    <row r="34" spans="1:22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:22" ht="16" customHeight="1" ns3:dyDescent="0.2">
       <c r="A34" s="8">
         <v>89</v>
       </c>
@@ -78733,7 +78779,7 @@
       <c r="U34" s="11"/>
       <c r="V34" s="11"/>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:22" ns3:dyDescent="0.2">
       <c r="A35" s="8">
         <v>94</v>
       </c>
@@ -78785,12 +78831,14 @@
       <c r="R35" t="s">
         <v>281</v>
       </c>
-      <c r="S35" s="11"/>
+      <c r="S35" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T35" s="10"/>
       <c r="U35" s="11"/>
       <c r="V35" s="11"/>
     </row>
-    <row r="36" spans="1:22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:22" ht="16" customHeight="1" ns3:dyDescent="0.2">
       <c r="A36" s="8">
         <v>100</v>
       </c>
@@ -78851,7 +78899,7 @@
       <c r="U36" s="11"/>
       <c r="V36" s="11"/>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:22" ns3:dyDescent="0.2">
       <c r="A37" s="8">
         <v>101</v>
       </c>
@@ -78912,7 +78960,7 @@
       <c r="U37" s="11"/>
       <c r="V37" s="11"/>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:22" ns3:dyDescent="0.2">
       <c r="A38" s="8">
         <v>103</v>
       </c>
@@ -78971,7 +79019,7 @@
       <c r="U38" s="11"/>
       <c r="V38" s="11"/>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:22" ns3:dyDescent="0.2">
       <c r="A39" s="8">
         <v>105</v>
       </c>
@@ -79032,7 +79080,7 @@
       <c r="U39" s="11"/>
       <c r="V39" s="11"/>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:22" ns3:dyDescent="0.2">
       <c r="A40" s="8">
         <v>110</v>
       </c>
@@ -79093,7 +79141,7 @@
       <c r="U40" s="11"/>
       <c r="V40" s="11"/>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:22" ns3:dyDescent="0.2">
       <c r="A41" s="8">
         <v>115</v>
       </c>
@@ -79143,12 +79191,14 @@
       <c r="R41" t="s">
         <v>345</v>
       </c>
-      <c r="S41" s="11"/>
+      <c r="S41" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T41" s="10"/>
       <c r="U41" s="11"/>
       <c r="V41" s="11"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:22" ns3:dyDescent="0.2">
       <c r="A42" s="8">
         <v>122</v>
       </c>
@@ -79209,7 +79259,7 @@
       <c r="U42" s="11"/>
       <c r="V42" s="11"/>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:22" ns3:dyDescent="0.2">
       <c r="A43" s="8">
         <v>127</v>
       </c>
@@ -79261,12 +79311,14 @@
       <c r="R43" t="s">
         <v>380</v>
       </c>
-      <c r="S43" s="11"/>
+      <c r="S43" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T43" s="10"/>
       <c r="U43" s="11"/>
       <c r="V43" s="11"/>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:22" ns3:dyDescent="0.2">
       <c r="A44" s="8">
         <v>128</v>
       </c>
@@ -79327,7 +79379,7 @@
       <c r="U44" s="11"/>
       <c r="V44" s="11"/>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:22" ns3:dyDescent="0.2">
       <c r="A45" s="8">
         <v>128</v>
       </c>
@@ -79388,7 +79440,7 @@
       <c r="U45" s="11"/>
       <c r="V45" s="11"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:22" ns3:dyDescent="0.2">
       <c r="A46" s="8">
         <v>128</v>
       </c>
@@ -79447,7 +79499,7 @@
       <c r="U46" s="11"/>
       <c r="V46" s="11"/>
     </row>
-    <row r="47" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:22" ht="16" ns3:dyDescent="0.2">
       <c r="A47" s="8">
         <v>130</v>
       </c>
@@ -79499,12 +79551,14 @@
       <c r="R47" s="72" t="s">
         <v>387</v>
       </c>
-      <c r="S47" s="11"/>
+      <c r="S47" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T47" s="10"/>
       <c r="U47" s="11"/>
       <c r="V47" s="11"/>
     </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:22" ns3:dyDescent="0.2">
       <c r="A48" s="8">
         <v>133</v>
       </c>
@@ -79563,7 +79617,7 @@
       <c r="U48" s="11"/>
       <c r="V48" s="11"/>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:22" ns3:dyDescent="0.2">
       <c r="A49" s="8">
         <v>142</v>
       </c>
@@ -79615,12 +79669,14 @@
       <c r="R49" t="s">
         <v>426</v>
       </c>
-      <c r="S49" s="11"/>
+      <c r="S49" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T49" s="10"/>
       <c r="U49" s="11"/>
       <c r="V49" s="11"/>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:22" ns3:dyDescent="0.2">
       <c r="A50" s="8">
         <v>144</v>
       </c>
@@ -79677,7 +79733,7 @@
       <c r="U50" s="11"/>
       <c r="V50" s="11"/>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:22" ns3:dyDescent="0.2">
       <c r="A51" s="8">
         <v>145</v>
       </c>
@@ -79734,7 +79790,7 @@
       <c r="U51" s="11"/>
       <c r="V51" s="11"/>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:22" ns3:dyDescent="0.2">
       <c r="A52" s="8">
         <v>146</v>
       </c>
@@ -79791,7 +79847,7 @@
       <c r="U52" s="11"/>
       <c r="V52" s="11"/>
     </row>
-    <row r="53" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:22" ht="16" ns3:dyDescent="0.2">
       <c r="A53" s="8">
         <v>150</v>
       </c>
@@ -79843,12 +79899,14 @@
       <c r="R53" s="72" t="s">
         <v>450</v>
       </c>
-      <c r="S53" s="11"/>
+      <c r="S53" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T53" s="10"/>
       <c r="U53" s="11"/>
       <c r="V53" s="11"/>
     </row>
-    <row r="54" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:22" ht="16" ns3:dyDescent="0.2">
       <c r="A54" s="8">
         <v>150</v>
       </c>
@@ -79898,12 +79956,14 @@
       <c r="R54" s="72" t="s">
         <v>450</v>
       </c>
-      <c r="S54" s="11"/>
+      <c r="S54" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T54" s="10"/>
       <c r="U54" s="11"/>
       <c r="V54" s="11"/>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:22" ns3:dyDescent="0.2">
       <c r="A55" s="8">
         <v>157</v>
       </c>
@@ -79962,7 +80022,7 @@
       <c r="U55" s="11"/>
       <c r="V55" s="11"/>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:22" ns3:dyDescent="0.2">
       <c r="A56" s="8">
         <v>181</v>
       </c>
@@ -80009,17 +80069,19 @@
         <v>6</v>
       </c>
       <c r="Q56" t="s">
-        <v>499</v>
+        <v>3005</v>
       </c>
       <c r="R56" t="s">
-        <v>500</v>
-      </c>
-      <c r="S56" s="11"/>
+        <v>3568</v>
+      </c>
+      <c r="S56" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T56" s="10"/>
       <c r="U56" s="11"/>
       <c r="V56" s="11"/>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:22" ns3:dyDescent="0.2">
       <c r="A57" s="8">
         <v>194</v>
       </c>
@@ -80078,7 +80140,7 @@
       <c r="U57" s="11"/>
       <c r="V57" s="11"/>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:22" ns3:dyDescent="0.2">
       <c r="A58" s="8">
         <v>199</v>
       </c>
@@ -80139,7 +80201,7 @@
       <c r="U58" s="11"/>
       <c r="V58" s="11"/>
     </row>
-    <row r="59" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:22" ht="16" ns3:dyDescent="0.2">
       <c r="A59" s="8">
         <v>208</v>
       </c>
@@ -80198,7 +80260,7 @@
       <c r="U59" s="11"/>
       <c r="V59" s="11"/>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:22" ns3:dyDescent="0.2">
       <c r="A60" s="8">
         <v>211</v>
       </c>
@@ -80259,7 +80321,7 @@
       <c r="U60" s="11"/>
       <c r="V60" s="11"/>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:22" ns3:dyDescent="0.2">
       <c r="A61" s="8">
         <v>212</v>
       </c>
@@ -80311,12 +80373,14 @@
       <c r="R61" t="s">
         <v>580</v>
       </c>
-      <c r="S61" s="11"/>
+      <c r="S61" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T61" s="10"/>
       <c r="U61" s="11"/>
       <c r="V61" s="11"/>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:22" ns3:dyDescent="0.2">
       <c r="A62" s="8">
         <v>214</v>
       </c>
@@ -80368,12 +80432,14 @@
       <c r="R62" t="s">
         <v>587</v>
       </c>
-      <c r="S62" s="11"/>
+      <c r="S62" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T62" s="10"/>
       <c r="U62" s="11"/>
       <c r="V62" s="11"/>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:22" ns3:dyDescent="0.2">
       <c r="A63" s="8">
         <v>215</v>
       </c>
@@ -80434,7 +80500,7 @@
       <c r="U63" s="11"/>
       <c r="V63" s="11"/>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:22" ns3:dyDescent="0.2">
       <c r="A64" s="8">
         <v>222</v>
       </c>
@@ -80491,7 +80557,7 @@
       <c r="U64" s="11"/>
       <c r="V64" s="11"/>
     </row>
-    <row r="65" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:22" ht="16" ns3:dyDescent="0.2">
       <c r="A65" s="8">
         <v>229</v>
       </c>
@@ -80543,12 +80609,14 @@
       <c r="R65" s="72" t="s">
         <v>624</v>
       </c>
-      <c r="S65" s="11"/>
+      <c r="S65" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T65" s="10"/>
       <c r="U65" s="11"/>
       <c r="V65" s="11"/>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:22" ns3:dyDescent="0.2">
       <c r="A66" s="8">
         <v>248</v>
       </c>
@@ -80600,12 +80668,14 @@
       <c r="R66" t="s">
         <v>659</v>
       </c>
-      <c r="S66" s="11"/>
+      <c r="S66" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T66" s="10"/>
       <c r="U66" s="11"/>
       <c r="V66" s="11"/>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:22" ns3:dyDescent="0.2">
       <c r="A67" s="8">
         <v>254</v>
       </c>
@@ -80657,12 +80727,14 @@
       <c r="R67" s="16" t="s">
         <v>673</v>
       </c>
-      <c r="S67" s="11"/>
+      <c r="S67" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T67" s="10"/>
       <c r="U67" s="11"/>
       <c r="V67" s="11"/>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:22" ns3:dyDescent="0.2">
       <c r="A68" s="8">
         <v>257</v>
       </c>
@@ -80714,12 +80786,14 @@
       <c r="R68" t="s">
         <v>678</v>
       </c>
-      <c r="S68" s="11"/>
+      <c r="S68" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T68" s="10"/>
       <c r="U68" s="11"/>
       <c r="V68" s="11"/>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:22" ns3:dyDescent="0.2">
       <c r="A69" s="8">
         <v>260</v>
       </c>
@@ -80771,12 +80845,14 @@
       <c r="R69" t="s">
         <v>683</v>
       </c>
-      <c r="S69" s="11"/>
+      <c r="S69" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T69" s="10"/>
       <c r="U69" s="11"/>
       <c r="V69" s="11"/>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:22" ns3:dyDescent="0.2">
       <c r="A70" s="8">
         <v>263</v>
       </c>
@@ -80837,7 +80913,7 @@
       <c r="U70" s="11"/>
       <c r="V70" s="11"/>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:22" ns3:dyDescent="0.2">
       <c r="A71" s="8">
         <v>264</v>
       </c>
@@ -80898,7 +80974,7 @@
       <c r="U71" s="11"/>
       <c r="V71" s="11"/>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:22" ns3:dyDescent="0.2">
       <c r="A72" s="8">
         <v>282</v>
       </c>
@@ -80950,12 +81026,14 @@
       <c r="R72" t="s">
         <v>2919</v>
       </c>
-      <c r="S72" s="11"/>
+      <c r="S72" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T72" s="10"/>
       <c r="U72" s="11"/>
       <c r="V72" s="11"/>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:22" ns3:dyDescent="0.2">
       <c r="A73" s="8">
         <v>302</v>
       </c>
@@ -81007,12 +81085,14 @@
       <c r="R73" t="s">
         <v>765</v>
       </c>
-      <c r="S73" s="11"/>
+      <c r="S73" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T73" s="10"/>
       <c r="U73" s="11"/>
       <c r="V73" s="11"/>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:22" ns3:dyDescent="0.2">
       <c r="A74" s="8">
         <v>303</v>
       </c>
@@ -81064,12 +81144,14 @@
       <c r="R74" t="s">
         <v>768</v>
       </c>
-      <c r="S74" s="11"/>
+      <c r="S74" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T74" s="10"/>
       <c r="U74" s="11"/>
       <c r="V74" s="11"/>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:22" ns3:dyDescent="0.2">
       <c r="A75" s="8">
         <v>306</v>
       </c>
@@ -81114,17 +81196,19 @@
         <v>6</v>
       </c>
       <c r="Q75" s="70" t="s">
-        <v>770</v>
+        <v>3010</v>
       </c>
       <c r="R75" t="s">
-        <v>771</v>
-      </c>
-      <c r="S75" s="11"/>
+        <v>3569</v>
+      </c>
+      <c r="S75" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T75" s="10"/>
       <c r="U75" s="11"/>
       <c r="V75" s="11"/>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:22" ns3:dyDescent="0.2">
       <c r="A76" s="8">
         <v>308</v>
       </c>
@@ -81176,12 +81260,14 @@
       <c r="R76" t="s">
         <v>777</v>
       </c>
-      <c r="S76" s="11"/>
+      <c r="S76" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T76" s="10"/>
       <c r="U76" s="11"/>
       <c r="V76" s="11"/>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:22" ns3:dyDescent="0.2">
       <c r="A77" s="8">
         <v>310</v>
       </c>
@@ -81226,17 +81312,19 @@
         <v>6</v>
       </c>
       <c r="Q77" t="s">
-        <v>781</v>
+        <v>3121</v>
       </c>
       <c r="R77" t="s">
-        <v>782</v>
-      </c>
-      <c r="S77" s="11"/>
+        <v>3570</v>
+      </c>
+      <c r="S77" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T77" s="10"/>
       <c r="U77" s="11"/>
       <c r="V77" s="11"/>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:22" ns3:dyDescent="0.2">
       <c r="A78" s="8">
         <v>319</v>
       </c>
@@ -81288,12 +81376,14 @@
       <c r="R78" t="s">
         <v>802</v>
       </c>
-      <c r="S78" s="11"/>
+      <c r="S78" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T78" s="10"/>
       <c r="U78" s="11"/>
       <c r="V78" s="11"/>
     </row>
-    <row r="79" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:22" ht="16" ns3:dyDescent="0.2">
       <c r="A79" s="8">
         <v>323</v>
       </c>
@@ -81344,12 +81434,14 @@
       <c r="R79" s="72" t="s">
         <v>811</v>
       </c>
-      <c r="S79" s="11"/>
+      <c r="S79" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T79" s="10"/>
       <c r="U79" s="11"/>
       <c r="V79" s="11"/>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:22" ns3:dyDescent="0.2">
       <c r="A80" s="8">
         <v>334</v>
       </c>
@@ -81401,12 +81493,14 @@
       <c r="R80" t="s">
         <v>835</v>
       </c>
-      <c r="S80" s="11"/>
+      <c r="S80" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T80" s="10"/>
       <c r="U80" s="11"/>
       <c r="V80" s="11"/>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:22" ns3:dyDescent="0.2">
       <c r="A81" s="8">
         <v>351</v>
       </c>
@@ -81461,7 +81555,7 @@
       <c r="U81" s="11"/>
       <c r="V81" s="11"/>
     </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:22" ns3:dyDescent="0.2">
       <c r="A82" s="8">
         <v>351</v>
       </c>
@@ -81516,7 +81610,7 @@
       <c r="U82" s="11"/>
       <c r="V82" s="11"/>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:22" ns3:dyDescent="0.2">
       <c r="A83" s="8">
         <v>351</v>
       </c>
@@ -81571,7 +81665,7 @@
       <c r="U83" s="11"/>
       <c r="V83" s="11"/>
     </row>
-    <row r="84" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:22" ns3:dyDescent="0.2">
       <c r="A84" s="8">
         <v>354</v>
       </c>
@@ -81621,12 +81715,14 @@
       <c r="R84" t="s">
         <v>884</v>
       </c>
-      <c r="S84" s="11"/>
+      <c r="S84" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T84" s="10"/>
       <c r="U84" s="11"/>
       <c r="V84" s="11"/>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:22" ns3:dyDescent="0.2">
       <c r="A85" s="8">
         <v>359</v>
       </c>
@@ -81676,12 +81772,14 @@
       <c r="R85" t="s">
         <v>896</v>
       </c>
-      <c r="S85" s="11"/>
+      <c r="S85" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T85" s="10"/>
       <c r="U85" s="11"/>
       <c r="V85" s="11"/>
     </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:22" ns3:dyDescent="0.2">
       <c r="A86" s="8">
         <v>362</v>
       </c>
@@ -81731,12 +81829,14 @@
       <c r="R86" t="s">
         <v>900</v>
       </c>
-      <c r="S86" s="11"/>
+      <c r="S86" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T86" s="10"/>
       <c r="U86" s="11"/>
       <c r="V86" s="11"/>
     </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:22" ns3:dyDescent="0.2">
       <c r="A87" s="8">
         <v>373</v>
       </c>
@@ -81783,17 +81883,19 @@
         <v>6</v>
       </c>
       <c r="Q87" s="70" t="s">
-        <v>916</v>
+        <v>3044</v>
       </c>
       <c r="R87" t="s">
-        <v>917</v>
-      </c>
-      <c r="S87" s="11"/>
+        <v>3571</v>
+      </c>
+      <c r="S87" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T87" s="10"/>
       <c r="U87" s="11"/>
       <c r="V87" s="11"/>
     </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:22" ns3:dyDescent="0.2">
       <c r="A88" s="8">
         <v>376</v>
       </c>
@@ -81845,12 +81947,14 @@
       <c r="R88" t="s">
         <v>922</v>
       </c>
-      <c r="S88" s="11"/>
+      <c r="S88" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T88" s="10"/>
       <c r="U88" s="11"/>
       <c r="V88" s="11"/>
     </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:22" ns3:dyDescent="0.2">
       <c r="A89" s="8">
         <v>380</v>
       </c>
@@ -81897,17 +82001,19 @@
         <v>6</v>
       </c>
       <c r="Q89" s="70" t="s">
-        <v>934</v>
+        <v>3048</v>
       </c>
       <c r="R89" t="s">
-        <v>935</v>
-      </c>
-      <c r="S89" s="11"/>
+        <v>3572</v>
+      </c>
+      <c r="S89" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T89" s="10"/>
       <c r="U89" s="11"/>
       <c r="V89" s="11"/>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:22" ns3:dyDescent="0.2">
       <c r="A90" s="8">
         <v>381</v>
       </c>
@@ -81954,17 +82060,19 @@
         <v>6</v>
       </c>
       <c r="Q90" s="70" t="s">
-        <v>937</v>
+        <v>3049</v>
       </c>
       <c r="R90" t="s">
-        <v>938</v>
-      </c>
-      <c r="S90" s="11"/>
+        <v>3573</v>
+      </c>
+      <c r="S90" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T90" s="10"/>
       <c r="U90" s="11"/>
       <c r="V90" s="11"/>
     </row>
-    <row r="91" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:22" ns3:dyDescent="0.2">
       <c r="A91" s="8">
         <v>382</v>
       </c>
@@ -82019,7 +82127,7 @@
       <c r="U91" s="11"/>
       <c r="V91" s="11"/>
     </row>
-    <row r="92" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:22" ns3:dyDescent="0.2">
       <c r="A92" s="8">
         <v>383</v>
       </c>
@@ -82076,7 +82184,7 @@
       <c r="U92" s="11"/>
       <c r="V92" s="11"/>
     </row>
-    <row r="93" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:22" ns3:dyDescent="0.2">
       <c r="A93" s="8">
         <v>384</v>
       </c>
@@ -82123,17 +82231,17 @@
         <v>6</v>
       </c>
       <c r="Q93" t="s">
-        <v>948</v>
+        <v>3574</v>
       </c>
       <c r="R93" t="s">
-        <v>949</v>
+        <v>3575</v>
       </c>
       <c r="S93" s="11"/>
       <c r="T93" s="10"/>
       <c r="U93" s="11"/>
       <c r="V93" s="11"/>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:22" ns3:dyDescent="0.2">
       <c r="A94" s="8">
         <v>386</v>
       </c>
@@ -82188,7 +82296,7 @@
       <c r="U94" s="11"/>
       <c r="V94" s="11"/>
     </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:22" ns3:dyDescent="0.2">
       <c r="A95" s="8">
         <v>386</v>
       </c>
@@ -82243,7 +82351,7 @@
       <c r="U95" s="11"/>
       <c r="V95" s="11"/>
     </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:22" ns3:dyDescent="0.2">
       <c r="A96" s="8">
         <v>386</v>
       </c>
@@ -82298,7 +82406,7 @@
       <c r="U96" s="11"/>
       <c r="V96" s="11"/>
     </row>
-    <row r="97" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:22" ht="16" ns3:dyDescent="0.2">
       <c r="A97" s="8">
         <v>412</v>
       </c>
@@ -82355,7 +82463,7 @@
       <c r="U97" s="11"/>
       <c r="V97" s="11"/>
     </row>
-    <row r="98" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:22" ht="16" ns3:dyDescent="0.2">
       <c r="A98" s="8">
         <v>412</v>
       </c>
@@ -82412,7 +82520,7 @@
       <c r="U98" s="11"/>
       <c r="V98" s="11"/>
     </row>
-    <row r="99" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:22" ht="16" ns3:dyDescent="0.2">
       <c r="A99" s="8">
         <v>413</v>
       </c>
@@ -82471,7 +82579,7 @@
       <c r="U99" s="11"/>
       <c r="V99" s="11"/>
     </row>
-    <row r="100" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:22" ht="16" ns3:dyDescent="0.2">
       <c r="A100" s="8">
         <v>413</v>
       </c>
@@ -82530,7 +82638,7 @@
       <c r="U100" s="11"/>
       <c r="V100" s="11"/>
     </row>
-    <row r="101" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:22" ns3:dyDescent="0.2">
       <c r="A101" s="8">
         <v>428</v>
       </c>
@@ -82582,12 +82690,14 @@
       <c r="R101" t="s">
         <v>1029</v>
       </c>
-      <c r="S101" s="11"/>
+      <c r="S101" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T101" s="10"/>
       <c r="U101" s="11"/>
       <c r="V101" s="11"/>
     </row>
-    <row r="102" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:22" ns3:dyDescent="0.2">
       <c r="A102" s="8">
         <v>445</v>
       </c>
@@ -82639,12 +82749,14 @@
       <c r="R102" t="s">
         <v>1056</v>
       </c>
-      <c r="S102" s="11"/>
+      <c r="S102" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T102" s="10"/>
       <c r="U102" s="11"/>
       <c r="V102" s="11"/>
     </row>
-    <row r="103" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:22" ns3:dyDescent="0.2">
       <c r="A103" s="8">
         <v>448</v>
       </c>
@@ -82696,12 +82808,14 @@
       <c r="R103" t="s">
         <v>1062</v>
       </c>
-      <c r="S103" s="11"/>
+      <c r="S103" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T103" s="10"/>
       <c r="U103" s="11"/>
       <c r="V103" s="11"/>
     </row>
-    <row r="104" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:22" ns3:dyDescent="0.2">
       <c r="A104" s="8">
         <v>460</v>
       </c>
@@ -82753,12 +82867,14 @@
       <c r="R104" t="s">
         <v>1087</v>
       </c>
-      <c r="S104" s="11"/>
+      <c r="S104" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T104" s="10"/>
       <c r="U104" s="11"/>
       <c r="V104" s="11"/>
     </row>
-    <row r="105" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:22" ns3:dyDescent="0.2">
       <c r="A105" s="8">
         <v>475</v>
       </c>
@@ -82810,12 +82926,14 @@
       <c r="R105" t="s">
         <v>1110</v>
       </c>
-      <c r="S105" s="11"/>
+      <c r="S105" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T105" s="10"/>
       <c r="U105" s="11"/>
       <c r="V105" s="11"/>
     </row>
-    <row r="106" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:22" ns3:dyDescent="0.2">
       <c r="A106" s="12">
         <v>479</v>
       </c>
@@ -82873,7 +82991,7 @@
       <c r="U106" s="11"/>
       <c r="V106" s="11"/>
     </row>
-    <row r="107" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:22" ns3:dyDescent="0.2">
       <c r="A107" s="12">
         <v>479</v>
       </c>
@@ -82932,7 +83050,7 @@
       <c r="U107" s="11"/>
       <c r="V107" s="11"/>
     </row>
-    <row r="108" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:22" ns3:dyDescent="0.2">
       <c r="A108" s="12">
         <v>479</v>
       </c>
@@ -82991,7 +83109,7 @@
       <c r="U108" s="11"/>
       <c r="V108" s="11"/>
     </row>
-    <row r="109" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:22" ns3:dyDescent="0.2">
       <c r="A109" s="12">
         <v>479</v>
       </c>
@@ -83050,7 +83168,7 @@
       <c r="U109" s="11"/>
       <c r="V109" s="11"/>
     </row>
-    <row r="110" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:22" ns3:dyDescent="0.2">
       <c r="A110" s="12">
         <v>479</v>
       </c>
@@ -83109,7 +83227,7 @@
       <c r="U110" s="11"/>
       <c r="V110" s="11"/>
     </row>
-    <row r="111" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:22" ns3:dyDescent="0.2">
       <c r="A111" s="8">
         <v>483</v>
       </c>
@@ -83168,7 +83286,7 @@
       <c r="U111" s="11"/>
       <c r="V111" s="11"/>
     </row>
-    <row r="112" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:22" ns3:dyDescent="0.2">
       <c r="A112" s="8">
         <v>484</v>
       </c>
@@ -83227,7 +83345,7 @@
       <c r="U112" s="11"/>
       <c r="V112" s="11"/>
     </row>
-    <row r="113" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:22" ns3:dyDescent="0.2">
       <c r="A113" s="8">
         <v>487</v>
       </c>
@@ -83284,7 +83402,7 @@
       <c r="U113" s="11"/>
       <c r="V113" s="11"/>
     </row>
-    <row r="114" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:22" ns3:dyDescent="0.2">
       <c r="A114" s="8">
         <v>492</v>
       </c>
@@ -83341,7 +83459,7 @@
       <c r="U114" s="11"/>
       <c r="V114" s="11"/>
     </row>
-    <row r="115" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:22" ns3:dyDescent="0.2">
       <c r="A115" s="8">
         <v>503</v>
       </c>
@@ -83400,7 +83518,7 @@
       <c r="U115" s="11"/>
       <c r="V115" s="11"/>
     </row>
-    <row r="116" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:22" ht="16" ns3:dyDescent="0.2">
       <c r="A116" s="8">
         <v>531</v>
       </c>
@@ -83452,12 +83570,14 @@
       <c r="R116" s="72" t="s">
         <v>2973</v>
       </c>
-      <c r="S116" s="11"/>
+      <c r="S116" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T116" s="10"/>
       <c r="U116" s="11"/>
       <c r="V116" s="11"/>
     </row>
-    <row r="117" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:22" ns3:dyDescent="0.2">
       <c r="A117" s="8">
         <v>549</v>
       </c>
@@ -83518,7 +83638,7 @@
       <c r="U117" s="11"/>
       <c r="V117" s="11"/>
     </row>
-    <row r="118" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:22" ns3:dyDescent="0.2">
       <c r="A118" s="8">
         <v>550</v>
       </c>
@@ -83577,7 +83697,7 @@
       <c r="U118" s="11"/>
       <c r="V118" s="11"/>
     </row>
-    <row r="119" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:22" ns3:dyDescent="0.2">
       <c r="A119" s="8">
         <v>550</v>
       </c>
@@ -83636,7 +83756,7 @@
       <c r="U119" s="11"/>
       <c r="V119" s="11"/>
     </row>
-    <row r="120" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:22" ns3:dyDescent="0.2">
       <c r="A120" s="8">
         <v>554</v>
       </c>
@@ -83693,7 +83813,7 @@
       <c r="U120" s="11"/>
       <c r="V120" s="11"/>
     </row>
-    <row r="121" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:22" ns3:dyDescent="0.2">
       <c r="A121" s="8">
         <v>555</v>
       </c>
@@ -83750,7 +83870,7 @@
       <c r="U121" s="11"/>
       <c r="V121" s="11"/>
     </row>
-    <row r="122" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:22" ns3:dyDescent="0.2">
       <c r="A122" s="8">
         <v>555</v>
       </c>
@@ -83809,7 +83929,7 @@
       <c r="U122" s="11"/>
       <c r="V122" s="11"/>
     </row>
-    <row r="123" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:22" ns3:dyDescent="0.2">
       <c r="A123" s="8">
         <v>555</v>
       </c>
@@ -83866,7 +83986,7 @@
       <c r="U123" s="11"/>
       <c r="V123" s="11"/>
     </row>
-    <row r="124" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:22" ns3:dyDescent="0.2">
       <c r="A124" s="8">
         <v>562</v>
       </c>
@@ -83923,7 +84043,7 @@
       <c r="U124" s="11"/>
       <c r="V124" s="11"/>
     </row>
-    <row r="125" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:22" ns3:dyDescent="0.2">
       <c r="A125" s="8">
         <v>570</v>
       </c>
@@ -83980,7 +84100,7 @@
       <c r="U125" s="11"/>
       <c r="V125" s="11"/>
     </row>
-    <row r="126" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:22" ns3:dyDescent="0.2">
       <c r="A126" s="8">
         <v>571</v>
       </c>
@@ -84037,7 +84157,7 @@
       <c r="U126" s="11"/>
       <c r="V126" s="11"/>
     </row>
-    <row r="127" spans="1:22" ht="16" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:22" ht="16" ns3:dyDescent="0.25">
       <c r="A127" s="8">
         <v>618</v>
       </c>
@@ -84094,7 +84214,7 @@
       <c r="U127" s="11"/>
       <c r="V127" s="11"/>
     </row>
-    <row r="128" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:22" ns3:dyDescent="0.2">
       <c r="A128" s="8">
         <v>628</v>
       </c>
@@ -84155,7 +84275,7 @@
       <c r="U128" s="11"/>
       <c r="V128" s="11"/>
     </row>
-    <row r="129" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:22" ns3:dyDescent="0.2">
       <c r="A129" s="8">
         <v>641</v>
       </c>
@@ -84210,7 +84330,7 @@
       <c r="U129" s="11"/>
       <c r="V129" s="11"/>
     </row>
-    <row r="130" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:22" ns3:dyDescent="0.2">
       <c r="A130" s="8">
         <v>642</v>
       </c>
@@ -84267,7 +84387,7 @@
       <c r="U130" s="11"/>
       <c r="V130" s="11"/>
     </row>
-    <row r="131" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:22" ns3:dyDescent="0.2">
       <c r="A131" s="8">
         <v>645</v>
       </c>
@@ -84324,7 +84444,7 @@
       <c r="U131" s="11"/>
       <c r="V131" s="11"/>
     </row>
-    <row r="132" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:22" ns3:dyDescent="0.2">
       <c r="A132" s="8">
         <v>646</v>
       </c>
@@ -84381,7 +84501,7 @@
       <c r="U132" s="11"/>
       <c r="V132" s="11"/>
     </row>
-    <row r="133" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:22" ns3:dyDescent="0.2">
       <c r="A133" s="8">
         <v>646</v>
       </c>
@@ -84438,7 +84558,7 @@
       <c r="U133" s="11"/>
       <c r="V133" s="11"/>
     </row>
-    <row r="134" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:22" ns3:dyDescent="0.2">
       <c r="A134" s="8">
         <v>647</v>
       </c>
@@ -84497,7 +84617,7 @@
       <c r="U134" s="11"/>
       <c r="V134" s="11"/>
     </row>
-    <row r="135" spans="1:22" ht="16" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:22" ht="16" ns3:dyDescent="0.25">
       <c r="A135" s="8">
         <v>648</v>
       </c>
@@ -84556,7 +84676,7 @@
       <c r="U135" s="11"/>
       <c r="V135" s="11"/>
     </row>
-    <row r="136" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:22" ns3:dyDescent="0.2">
       <c r="A136" s="8">
         <v>658</v>
       </c>
@@ -84613,7 +84733,7 @@
       <c r="U136" s="11"/>
       <c r="V136" s="11"/>
     </row>
-    <row r="137" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:22" ns3:dyDescent="0.2">
       <c r="A137" s="8">
         <v>678</v>
       </c>
@@ -84672,7 +84792,7 @@
       <c r="U137" s="11"/>
       <c r="V137" s="11"/>
     </row>
-    <row r="138" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:22" ns3:dyDescent="0.2">
       <c r="A138" s="8">
         <v>681</v>
       </c>
@@ -84729,7 +84849,7 @@
       <c r="U138" s="11"/>
       <c r="V138" s="11"/>
     </row>
-    <row r="139" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:22" ns3:dyDescent="0.2">
       <c r="A139" s="8">
         <v>705</v>
       </c>
@@ -84790,7 +84910,7 @@
       <c r="U139" s="11"/>
       <c r="V139" s="11"/>
     </row>
-    <row r="140" spans="1:22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:22" ht="16" customHeight="1" ns3:dyDescent="0.2">
       <c r="A140" s="8">
         <v>706</v>
       </c>
@@ -84851,7 +84971,7 @@
       <c r="U140" s="11"/>
       <c r="V140" s="11"/>
     </row>
-    <row r="141" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:22" ns3:dyDescent="0.2">
       <c r="A141" s="8">
         <v>710</v>
       </c>
@@ -84912,7 +85032,7 @@
       <c r="U141" s="11"/>
       <c r="V141" s="11"/>
     </row>
-    <row r="142" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:22" ns3:dyDescent="0.2">
       <c r="A142" s="8">
         <v>710</v>
       </c>
@@ -84973,7 +85093,7 @@
       <c r="U142" s="11"/>
       <c r="V142" s="11"/>
     </row>
-    <row r="143" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:22" ns3:dyDescent="0.2">
       <c r="A143" s="8">
         <v>710</v>
       </c>
@@ -85034,7 +85154,7 @@
       <c r="U143" s="11"/>
       <c r="V143" s="11"/>
     </row>
-    <row r="144" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:22" ns3:dyDescent="0.2">
       <c r="A144" s="8">
         <v>711</v>
       </c>
@@ -85095,7 +85215,7 @@
       <c r="U144" s="11"/>
       <c r="V144" s="11"/>
     </row>
-    <row r="145" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:22" ns3:dyDescent="0.2">
       <c r="A145" s="8">
         <v>711</v>
       </c>
@@ -85156,7 +85276,7 @@
       <c r="U145" s="11"/>
       <c r="V145" s="11"/>
     </row>
-    <row r="146" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:22" ns3:dyDescent="0.2">
       <c r="A146" s="8">
         <v>711</v>
       </c>
@@ -85217,7 +85337,7 @@
       <c r="U146" s="11"/>
       <c r="V146" s="11"/>
     </row>
-    <row r="147" spans="1:22" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:22" ht="19" customHeight="1" ns3:dyDescent="0.2">
       <c r="A147" s="12">
         <v>713</v>
       </c>
@@ -85278,7 +85398,7 @@
       <c r="U147" s="11"/>
       <c r="V147" s="11"/>
     </row>
-    <row r="148" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:22" ht="16" ns3:dyDescent="0.2">
       <c r="A148" s="8">
         <v>718</v>
       </c>
@@ -85335,7 +85455,7 @@
       <c r="U148" s="11"/>
       <c r="V148" s="11"/>
     </row>
-    <row r="149" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:22" ht="16" ns3:dyDescent="0.2">
       <c r="A149" s="8">
         <v>718</v>
       </c>
@@ -85392,7 +85512,7 @@
       <c r="U149" s="11"/>
       <c r="V149" s="11"/>
     </row>
-    <row r="150" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:22" ns3:dyDescent="0.2">
       <c r="A150" s="8">
         <v>719</v>
       </c>
@@ -85444,12 +85564,14 @@
       <c r="R150" t="s">
         <v>1595</v>
       </c>
-      <c r="S150" s="11"/>
+      <c r="S150" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="T150" s="10"/>
       <c r="U150" s="11"/>
       <c r="V150" s="11"/>
     </row>
-    <row r="151" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:22" ns3:dyDescent="0.2">
       <c r="A151" s="8">
         <v>720</v>
       </c>
@@ -85506,7 +85628,7 @@
       <c r="U151" s="11"/>
       <c r="V151" s="11"/>
     </row>
-    <row r="152" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:22" ns3:dyDescent="0.2">
       <c r="A152" s="8">
         <v>724</v>
       </c>
@@ -85565,7 +85687,7 @@
       <c r="U152" s="11"/>
       <c r="V152" s="11"/>
     </row>
-    <row r="153" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:22" ns3:dyDescent="0.2">
       <c r="A153" s="8">
         <v>741</v>
       </c>
@@ -85622,7 +85744,7 @@
       <c r="U153" s="11"/>
       <c r="V153" s="11"/>
     </row>
-    <row r="154" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:22" ns3:dyDescent="0.2">
       <c r="A154" s="8">
         <v>741</v>
       </c>
@@ -85679,7 +85801,7 @@
       <c r="U154" s="11"/>
       <c r="V154" s="11"/>
     </row>
-    <row r="155" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:22" ns3:dyDescent="0.2">
       <c r="A155" s="8">
         <v>741</v>
       </c>
@@ -85736,7 +85858,7 @@
       <c r="U155" s="11"/>
       <c r="V155" s="11"/>
     </row>
-    <row r="156" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:22" ns3:dyDescent="0.2">
       <c r="A156" s="8">
         <v>744</v>
       </c>
@@ -85791,7 +85913,7 @@
       <c r="U156" s="11"/>
       <c r="V156" s="11"/>
     </row>
-    <row r="157" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:22" ns3:dyDescent="0.2">
       <c r="A157" s="8">
         <v>745</v>
       </c>
@@ -85846,7 +85968,7 @@
       <c r="U157" s="11"/>
       <c r="V157" s="11"/>
     </row>
-    <row r="158" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:22" ns3:dyDescent="0.2">
       <c r="A158" s="8">
         <v>745</v>
       </c>
@@ -85905,7 +86027,7 @@
       <c r="U158" s="11"/>
       <c r="V158" s="11"/>
     </row>
-    <row r="159" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:22" ns3:dyDescent="0.2">
       <c r="A159" s="8">
         <v>746</v>
       </c>
@@ -85960,7 +86082,7 @@
       <c r="U159" s="11"/>
       <c r="V159" s="11"/>
     </row>
-    <row r="160" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:22" ns3:dyDescent="0.2">
       <c r="A160" s="8">
         <v>774</v>
       </c>
@@ -86017,7 +86139,7 @@
       <c r="U160" s="11"/>
       <c r="V160" s="11"/>
     </row>
-    <row r="161" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:22" ns3:dyDescent="0.2">
       <c r="A161" s="8">
         <v>800</v>
       </c>
@@ -86074,7 +86196,7 @@
       <c r="U161" s="11"/>
       <c r="V161" s="11"/>
     </row>
-    <row r="162" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:22" ns3:dyDescent="0.2">
       <c r="A162" s="8">
         <v>800</v>
       </c>
@@ -86131,7 +86253,7 @@
       <c r="U162" s="11"/>
       <c r="V162" s="11"/>
     </row>
-    <row r="163" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:22" ns3:dyDescent="0.2">
       <c r="A163" s="8">
         <v>800</v>
       </c>
@@ -86188,7 +86310,7 @@
       <c r="U163" s="11"/>
       <c r="V163" s="11"/>
     </row>
-    <row r="164" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:22" ns3:dyDescent="0.2">
       <c r="A164" s="8">
         <v>849</v>
       </c>
@@ -86249,7 +86371,7 @@
       <c r="U164" s="11"/>
       <c r="V164" s="11"/>
     </row>
-    <row r="165" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:22" ns3:dyDescent="0.2">
       <c r="A165" s="8">
         <v>875</v>
       </c>
@@ -86304,7 +86426,7 @@
       <c r="U165" s="11"/>
       <c r="V165" s="11"/>
     </row>
-    <row r="166" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:22" ns3:dyDescent="0.2">
       <c r="A166" s="8">
         <v>876</v>
       </c>
@@ -86365,7 +86487,7 @@
       <c r="U166" s="11"/>
       <c r="V166" s="11"/>
     </row>
-    <row r="167" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:22" ns3:dyDescent="0.2">
       <c r="A167" s="8">
         <v>877</v>
       </c>
@@ -86422,7 +86544,7 @@
       <c r="U167" s="11"/>
       <c r="V167" s="11"/>
     </row>
-    <row r="168" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:22" ns3:dyDescent="0.2">
       <c r="A168" s="8">
         <v>888</v>
       </c>
@@ -86479,7 +86601,7 @@
       <c r="U168" s="11"/>
       <c r="V168" s="11"/>
     </row>
-    <row r="169" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:22" ns3:dyDescent="0.2">
       <c r="A169" s="8">
         <v>889</v>
       </c>
@@ -86536,7 +86658,7 @@
       <c r="U169" s="11"/>
       <c r="V169" s="11"/>
     </row>
-    <row r="170" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:22" ns3:dyDescent="0.2">
       <c r="A170" s="8">
         <v>890</v>
       </c>
@@ -86593,7 +86715,7 @@
       <c r="U170" s="11"/>
       <c r="V170" s="11"/>
     </row>
-    <row r="171" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:22" ns3:dyDescent="0.2">
       <c r="A171" s="8">
         <v>892</v>
       </c>
@@ -86650,7 +86772,7 @@
       <c r="U171" s="11"/>
       <c r="V171" s="11"/>
     </row>
-    <row r="172" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:22" ns3:dyDescent="0.2">
       <c r="A172" s="8">
         <v>898</v>
       </c>
@@ -86707,7 +86829,7 @@
       <c r="U172" s="11"/>
       <c r="V172" s="11"/>
     </row>
-    <row r="173" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:22" ns3:dyDescent="0.2">
       <c r="A173" s="8">
         <v>898</v>
       </c>
@@ -86764,7 +86886,7 @@
       <c r="U173" s="11"/>
       <c r="V173" s="11"/>
     </row>
-    <row r="174" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:22" ns3:dyDescent="0.2">
       <c r="A174" s="8">
         <v>901</v>
       </c>
@@ -86818,7 +86940,7 @@
       <c r="U174" s="11"/>
       <c r="V174" s="11"/>
     </row>
-    <row r="175" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:22" ns3:dyDescent="0.2">
       <c r="A175" s="8">
         <v>902</v>
       </c>
@@ -86879,7 +87001,7 @@
       <c r="U175" s="11"/>
       <c r="V175" s="11"/>
     </row>
-    <row r="176" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:22" ns3:dyDescent="0.2">
       <c r="A176" s="8">
         <v>905</v>
       </c>
@@ -86936,7 +87058,7 @@
       <c r="U176" s="11"/>
       <c r="V176" s="11"/>
     </row>
-    <row r="177" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:22" ns3:dyDescent="0.2">
       <c r="A177" s="8">
         <v>916</v>
       </c>
@@ -86995,7 +87117,7 @@
       <c r="U177" s="11"/>
       <c r="V177" s="11"/>
     </row>
-    <row r="178" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:22" ns3:dyDescent="0.2">
       <c r="A178" s="8">
         <v>925</v>
       </c>
@@ -87054,7 +87176,7 @@
       <c r="U178" s="11"/>
       <c r="V178" s="11"/>
     </row>
-    <row r="179" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:22" ns3:dyDescent="0.2">
       <c r="A179" s="8">
         <v>931</v>
       </c>
@@ -87115,7 +87237,7 @@
       <c r="U179" s="11"/>
       <c r="V179" s="11"/>
     </row>
-    <row r="180" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:22" ns3:dyDescent="0.2">
       <c r="A180" s="8">
         <v>931</v>
       </c>
@@ -87176,7 +87298,7 @@
       <c r="U180" s="11"/>
       <c r="V180" s="11"/>
     </row>
-    <row r="181" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:22" ns3:dyDescent="0.2">
       <c r="A181" s="8">
         <v>931</v>
       </c>
@@ -87237,7 +87359,7 @@
       <c r="U181" s="11"/>
       <c r="V181" s="11"/>
     </row>
-    <row r="182" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:22" ns3:dyDescent="0.2">
       <c r="A182" s="8">
         <v>964</v>
       </c>
@@ -87292,7 +87414,7 @@
       <c r="U182" s="11"/>
       <c r="V182" s="11"/>
     </row>
-    <row r="183" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:22" ns3:dyDescent="0.2">
       <c r="A183" s="8">
         <v>978</v>
       </c>
@@ -87351,7 +87473,7 @@
       <c r="U183" s="11"/>
       <c r="V183" s="11"/>
     </row>
-    <row r="184" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:22" ns3:dyDescent="0.2">
       <c r="A184" s="8">
         <v>978</v>
       </c>
@@ -87410,7 +87532,7 @@
       <c r="U184" s="11"/>
       <c r="V184" s="11"/>
     </row>
-    <row r="185" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:22" ns3:dyDescent="0.2">
       <c r="A185" s="8">
         <v>982</v>
       </c>
@@ -87469,7 +87591,7 @@
       <c r="U185" s="11"/>
       <c r="V185" s="11"/>
     </row>
-    <row r="186" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:22" ns3:dyDescent="0.2">
       <c r="A186" s="8">
         <v>999</v>
       </c>
@@ -87524,7 +87646,7 @@
       <c r="U186" s="11"/>
       <c r="V186" s="11"/>
     </row>
-    <row r="187" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:22" ns3:dyDescent="0.2">
       <c r="A187" s="8">
         <v>1017</v>
       </c>
@@ -87581,7 +87703,7 @@
       <c r="U187" s="11"/>
       <c r="V187" s="11"/>
     </row>
-    <row r="188" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:22" ns3:dyDescent="0.2">
       <c r="A188" s="8">
         <v>1017</v>
       </c>
@@ -87638,7 +87760,7 @@
       <c r="U188" s="11"/>
       <c r="V188" s="11"/>
     </row>
-    <row r="189" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:22" ns3:dyDescent="0.2">
       <c r="A189" s="8">
         <v>1017</v>
       </c>
@@ -87695,7 +87817,7 @@
       <c r="U189" s="11"/>
       <c r="V189" s="11"/>
     </row>
-    <row r="190" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:22" ht="16" ns3:dyDescent="0.2">
       <c r="A190" s="8">
         <v>1024</v>
       </c>
@@ -87750,7 +87872,7 @@
       <c r="U190" s="11"/>
       <c r="V190" s="11"/>
     </row>
-    <row r="191" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:22" ht="16" ns3:dyDescent="0.2">
       <c r="A191" s="8">
         <v>1024</v>
       </c>

</xml_diff>